<commit_message>
Frontend integrated and working
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vibek\OneDrive\Desktop\CSTec-Infosolutions-Assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B63D647-CB1C-4AD0-95A9-4E85F1374C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBEDB03-EB75-4B09-A6A9-C3EFF0A749B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>FirstName</t>
   </si>
@@ -33,25 +33,31 @@
     <t>Phone</t>
   </si>
   <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>Interested</t>
   </si>
   <si>
     <t>Rohan</t>
   </si>
   <si>
-    <t>Subham</t>
-  </si>
-  <si>
-    <t>Abhisek</t>
-  </si>
-  <si>
     <t>Callback</t>
   </si>
   <si>
-    <t>No Interested</t>
-  </si>
-  <si>
-    <t>Reviews</t>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>Shyam</t>
+  </si>
+  <si>
+    <t>Abhinash</t>
+  </si>
+  <si>
+    <t>Not Interested</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
 </sst>
 </file>
@@ -369,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.109375" customWidth="1"/>
@@ -385,40 +391,51 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>123456789</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>1234567890</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>1234567890</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>325652365</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>